<commit_message>
Fix Offline Transaction Import logic and template
- Handle robust date parsing for slash and dash formats

- Populate Target Duration from md_truck to calculate Target Status correctly

- Insert Activity Log for manually imported Offline Txs

- Translate error controller outputs

- Add non-strict Example row skipping mechanism
</commit_message>
<xml_diff>
--- a/public/exports/offline_import_template.xlsx
+++ b/public/exports/offline_import_template.xlsx
@@ -327,13 +327,13 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>unplanned</t>
-  </si>
-  <si>
-    <t>inbound</t>
-  </si>
-  <si>
-    <t>CDD/CDE</t>
+    <t>Example: unplanned</t>
+  </si>
+  <si>
+    <t>Example: inbound</t>
+  </si>
+  <si>
+    <t>Example: CDD/CDE</t>
   </si>
   <si>
     <t>15-04-2026 08:00</t>
@@ -345,7 +345,7 @@
     <t>15-04-2026 10:00</t>
   </si>
   <si>
-    <t>POC-12345</t>
+    <t>Example: POC-12345</t>
   </si>
   <si>
     <t>SJ-6829316</t>

</xml_diff>

<commit_message>
feat: vendor portal & reporting enhancements including offline import refactor, dashboard reporting metrics fix, vendor internal distinction, and UI layout fixes
</commit_message>
<xml_diff>
--- a/public/exports/offline_import_template.xlsx
+++ b/public/exports/offline_import_template.xlsx
@@ -135,7 +135,7 @@
             <u val="none"/>
           </rPr>
           <t xml:space="preserve">Wajib diisi
-Nomor PO/DO</t>
+Nomor PO/SO</t>
         </r>
       </text>
     </comment>
@@ -254,7 +254,7 @@
             <u val="none"/>
           </rPr>
           <t xml:space="preserve">Wajib diisi
-Pilihan: A,B,C</t>
+Pilihan: 1,2,3</t>
         </r>
       </text>
     </comment>
@@ -280,7 +280,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
   <si>
     <t>Slot Type *</t>
   </si>
@@ -345,7 +345,7 @@
     <t>15-04-2026 10:00</t>
   </si>
   <si>
-    <t>Example: POC-12345</t>
+    <t>Example: 1100001234</t>
   </si>
   <si>
     <t>SJ-6829316</t>
@@ -364,9 +364,6 @@
   </si>
   <si>
     <t>WH1</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
   <si>
     <t>Recorded during power outage</t>
@@ -898,11 +895,11 @@
       <c r="M2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="3">
+        <v>1</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -1606,7 +1603,7 @@
       <formula1>"WH1,WH2"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Invalid" error="Select gate number" sqref="N2:N100">
-      <formula1>"A,B,C"</formula1>
+      <formula1>"1,2,3"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>